<commit_message>
#6 L2 Change in Design and Deliverables Generated.
</commit_message>
<xml_diff>
--- a/Design_Files/Deliverables/BOM/BOM.xlsx
+++ b/Design_Files/Deliverables/BOM/BOM.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20409"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\antonmeyer-pcbtroubleshoot\Design_Files\Project Outputs for ESP32-C3FH4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\antonmeyer-pcbtroubleshoot\Design_Files\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C9DC1D-F69A-411A-9F87-BFFBA2D0CFCC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="128">
   <si>
     <t>#</t>
   </si>
@@ -221,9 +220,6 @@
     <t>TSW SMD-6*6*5</t>
   </si>
   <si>
-    <t>IND_CLF7045T-3R3N-D</t>
-  </si>
-  <si>
     <t>LED 0603B</t>
   </si>
   <si>
@@ -353,9 +349,6 @@
     <t>6*6*5</t>
   </si>
   <si>
-    <t>CLF7045T-3R3N-D</t>
-  </si>
-  <si>
     <t>GREEN</t>
   </si>
   <si>
@@ -408,12 +401,15 @@
   </si>
   <si>
     <t>Fuse</t>
+  </si>
+  <si>
+    <t>VLS5045EX-3R3N</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -692,14 +688,14 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -986,7 +982,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1011,8 +1007,8 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1032,16 +1028,16 @@
         <v>57</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1065,7 +1061,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="15"/>
       <c r="I3" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J3" s="15">
         <v>11</v>
@@ -1092,7 +1088,7 @@
       <c r="G4" s="18"/>
       <c r="H4" s="17"/>
       <c r="I4" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J4" s="17">
         <v>2</v>
@@ -1119,7 +1115,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="15"/>
       <c r="I5" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J5" s="15">
         <v>1</v>
@@ -1146,7 +1142,7 @@
       <c r="G6" s="18"/>
       <c r="H6" s="17"/>
       <c r="I6" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J6" s="17">
         <v>1</v>
@@ -1172,10 +1168,10 @@
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J7" s="15">
         <v>1</v>
@@ -1201,10 +1197,10 @@
       </c>
       <c r="G8" s="18"/>
       <c r="H8" s="17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J8" s="17">
         <v>1</v>
@@ -1231,7 +1227,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="15"/>
       <c r="I9" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J9" s="15">
         <v>1</v>
@@ -1257,10 +1253,10 @@
       </c>
       <c r="G10" s="18"/>
       <c r="H10" s="17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I10" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J10" s="17">
         <v>1</v>
@@ -1287,7 +1283,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="15"/>
       <c r="I11" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J11" s="15">
         <v>1</v>
@@ -1299,14 +1295,14 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>123</v>
+      <c r="C12" s="22" t="s">
+        <v>121</v>
       </c>
       <c r="D12" s="17" t="s">
         <v>18</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>60</v>
@@ -1314,7 +1310,7 @@
       <c r="G12" s="18"/>
       <c r="H12" s="17"/>
       <c r="I12" s="18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J12" s="17">
         <v>3</v>
@@ -1326,24 +1322,24 @@
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
-      <c r="C13" s="24" t="s">
-        <v>128</v>
+      <c r="C13" s="23" t="s">
+        <v>126</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F13" s="15" t="s">
         <v>61</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J13" s="15">
         <v>1</v>
@@ -1355,8 +1351,8 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="23" t="s">
-        <v>127</v>
+      <c r="C14" s="22" t="s">
+        <v>125</v>
       </c>
       <c r="D14" s="17" t="s">
         <v>20</v>
@@ -1370,7 +1366,7 @@
       <c r="G14" s="18"/>
       <c r="H14" s="17"/>
       <c r="I14" s="18" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J14" s="17">
         <v>1</v>
@@ -1382,8 +1378,8 @@
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="23" t="s">
-        <v>127</v>
+      <c r="C15" s="22" t="s">
+        <v>125</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>21</v>
@@ -1397,7 +1393,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="15"/>
       <c r="I15" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J15" s="15">
         <v>1</v>
@@ -1409,7 +1405,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="22" t="s">
         <v>2</v>
       </c>
       <c r="D16" s="17" t="s">
@@ -1422,13 +1418,13 @@
         <v>64</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I16" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J16" s="17">
         <v>1</v>
@@ -1440,8 +1436,8 @@
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="24" t="s">
-        <v>126</v>
+      <c r="C17" s="23" t="s">
+        <v>124</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>23</v>
@@ -1455,7 +1451,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="15"/>
       <c r="I17" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J17" s="15">
         <v>1</v>
@@ -1467,22 +1463,22 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="23" t="s">
-        <v>125</v>
+      <c r="C18" s="22" t="s">
+        <v>123</v>
       </c>
       <c r="D18" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="23" t="s">
-        <v>125</v>
+      <c r="E18" s="22" t="s">
+        <v>123</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>66</v>
+        <v>127</v>
       </c>
       <c r="G18" s="18"/>
       <c r="H18" s="17"/>
       <c r="I18" s="18" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="J18" s="17">
         <v>1</v>
@@ -1494,8 +1490,8 @@
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
-      <c r="C19" s="23" t="s">
-        <v>123</v>
+      <c r="C19" s="22" t="s">
+        <v>121</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>25</v>
@@ -1504,12 +1500,12 @@
         <v>47</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="15"/>
       <c r="I19" s="16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J19" s="15">
         <v>1</v>
@@ -1521,24 +1517,24 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C20" s="23" t="s">
-        <v>124</v>
+      <c r="C20" s="22" t="s">
+        <v>122</v>
       </c>
       <c r="D20" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="23" t="s">
-        <v>124</v>
+      <c r="E20" s="22" t="s">
+        <v>122</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G20" s="18"/>
       <c r="H20" s="17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I20" s="18" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="J20" s="17">
         <v>2</v>
@@ -1550,22 +1546,22 @@
         <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G21" s="16"/>
       <c r="H21" s="15"/>
       <c r="I21" s="16" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J21" s="15">
         <v>1</v>
@@ -1577,22 +1573,22 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D22" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G22" s="18"/>
       <c r="H22" s="17"/>
       <c r="I22" s="18" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J22" s="17">
         <v>6</v>
@@ -1604,22 +1600,22 @@
         <f>ROW(B23) - ROW($B$2)</f>
         <v>21</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="23" t="s">
+      <c r="E23" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G23" s="16"/>
       <c r="H23" s="15"/>
       <c r="I23" s="16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J23" s="15">
         <v>1</v>
@@ -1631,7 +1627,7 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D24" s="17" t="s">
@@ -1641,16 +1637,16 @@
         <v>48</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I24" s="18" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J24" s="17">
         <v>2</v>
@@ -1662,22 +1658,22 @@
         <f>ROW(B25) - ROW($B$2)</f>
         <v>23</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="E25" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="15"/>
       <c r="I25" s="16" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J25" s="15">
         <v>1</v>
@@ -1689,7 +1685,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D26" s="17" t="s">
@@ -1699,16 +1695,16 @@
         <v>49</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G26" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H26" s="17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I26" s="18" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J26" s="17">
         <v>1</v>
@@ -1720,7 +1716,7 @@
         <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="23" t="s">
         <v>5</v>
       </c>
       <c r="D27" s="15" t="s">
@@ -1730,12 +1726,12 @@
         <v>50</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G27" s="16"/>
       <c r="H27" s="15"/>
       <c r="I27" s="16" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J27" s="15">
         <v>1</v>
@@ -1747,7 +1743,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="23" t="s">
         <v>5</v>
       </c>
       <c r="D28" s="17" t="s">
@@ -1755,12 +1751,12 @@
       </c>
       <c r="E28" s="18"/>
       <c r="F28" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G28" s="18"/>
       <c r="H28" s="17"/>
       <c r="I28" s="18" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J28" s="17">
         <v>1</v>
@@ -1772,7 +1768,7 @@
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="23" t="s">
         <v>4</v>
       </c>
       <c r="D29" s="15" t="s">
@@ -1782,16 +1778,16 @@
         <v>51</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J29" s="15">
         <v>1</v>
@@ -1803,7 +1799,7 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C30" s="24" t="s">
+      <c r="C30" s="23" t="s">
         <v>5</v>
       </c>
       <c r="D30" s="17" t="s">
@@ -1813,12 +1809,12 @@
         <v>52</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G30" s="18"/>
       <c r="H30" s="17"/>
       <c r="I30" s="18" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J30" s="17">
         <v>1</v>
@@ -1830,7 +1826,7 @@
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
-      <c r="C31" s="24" t="s">
+      <c r="C31" s="23" t="s">
         <v>5</v>
       </c>
       <c r="D31" s="15" t="s">
@@ -1840,16 +1836,16 @@
         <v>53</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J31" s="15">
         <v>1</v>
@@ -1861,7 +1857,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="23" t="s">
         <v>5</v>
       </c>
       <c r="D32" s="17" t="s">
@@ -1871,12 +1867,12 @@
         <v>54</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G32" s="18"/>
       <c r="H32" s="17"/>
       <c r="I32" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J32" s="17">
         <v>1</v>
@@ -1888,7 +1884,7 @@
         <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
-      <c r="C33" s="24" t="s">
+      <c r="C33" s="23" t="s">
         <v>6</v>
       </c>
       <c r="D33" s="15" t="s">
@@ -1898,16 +1894,16 @@
         <v>55</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J33" s="15">
         <v>1</v>
@@ -1919,7 +1915,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="23" t="s">
+      <c r="C34" s="22" t="s">
         <v>7</v>
       </c>
       <c r="D34" s="17" t="s">
@@ -1929,16 +1925,16 @@
         <v>56</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I34" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J34" s="17">
         <v>1</v>

</xml_diff>